<commit_message>
Avances 07 de Septiembre 2026
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES 2.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88E36AD-92FE-461A-A5C0-830F7A1D2B4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF6F658-FC35-45DA-A962-0D847F5E8D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="0" windowWidth="36825" windowHeight="20880" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="179">
   <si>
     <t>Director(es) que lo solicita</t>
   </si>
@@ -598,9 +598,6 @@
     <t>Explicar los elementos de las ecuaciones presentes en la 2.5</t>
   </si>
   <si>
-    <t>Mencionar explicitamente la ecuiación del QDA, referenciarla en el texto y definir las variables.</t>
-  </si>
-  <si>
     <t>Eliminar los parentesis de las ecuaciones en la redacción</t>
   </si>
   <si>
@@ -692,13 +689,31 @@
   </si>
   <si>
     <t>Cambiar por Conclusiones y trabajo futuro</t>
+  </si>
+  <si>
+    <t>TIPO</t>
+  </si>
+  <si>
+    <t>FONDO</t>
+  </si>
+  <si>
+    <t>FORMA</t>
+  </si>
+  <si>
+    <t>Solicitante</t>
+  </si>
+  <si>
+    <t>Mencionar explicitamente la ecuación del QDA, referenciarla en el texto y definir las variables.</t>
+  </si>
+  <si>
+    <t>LISTO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -779,6 +794,14 @@
       <name val="Aptos"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -812,7 +835,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -850,11 +873,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -901,307 +935,23 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="34">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1534,15 +1284,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="33.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1556,7 +1306,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1570,7 +1320,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1584,7 +1334,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1598,7 +1348,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1612,7 +1362,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1626,7 +1376,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -1640,7 +1390,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -1654,7 +1404,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -1668,7 +1418,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -1682,7 +1432,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1696,7 +1446,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -1710,7 +1460,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>1</v>
       </c>
@@ -1724,7 +1474,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -1738,7 +1488,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1752,7 +1502,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -1766,7 +1516,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>20</v>
       </c>
@@ -1780,7 +1530,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>22</v>
       </c>
@@ -1794,7 +1544,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>1</v>
       </c>
@@ -1806,7 +1556,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>33</v>
       </c>
@@ -1820,7 +1570,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1832,7 +1582,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>4</v>
       </c>
@@ -1844,7 +1594,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -1856,7 +1606,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
@@ -1870,17 +1620,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A13 C13:D13">
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>$D$2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:D12">
-    <cfRule type="cellIs" dxfId="32" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
       <formula>$D$2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14:D24">
-    <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>$D$2</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1891,12 +1641,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8E058B-C30B-45F0-BBCF-B7D4D02421F4}">
   <dimension ref="B2:L12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>83</v>
       </c>
@@ -1928,7 +1678,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>88</v>
       </c>
@@ -1960,7 +1710,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4" s="18" t="s">
         <v>90</v>
       </c>
@@ -1992,7 +1742,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>92</v>
       </c>
@@ -2024,7 +1774,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>101</v>
       </c>
@@ -2056,7 +1806,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>95</v>
       </c>
@@ -2088,7 +1838,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="17" t="s">
         <v>97</v>
       </c>
@@ -2120,7 +1870,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>99</v>
       </c>
@@ -2152,7 +1902,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H10" s="18" t="s">
         <v>117</v>
       </c>
@@ -2169,7 +1919,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H11" t="s">
         <v>119</v>
       </c>
@@ -2186,7 +1936,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H12" t="s">
         <v>119</v>
       </c>
@@ -2211,12 +1961,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CD9C86-BB81-45D2-B52F-9BBB3BE4D29C}">
   <dimension ref="B2:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="46.5703125" customWidth="1"/>
+    <col min="4" max="4" width="46.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -2227,7 +1977,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>45</v>
       </c>
@@ -2238,7 +1988,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>45</v>
       </c>
@@ -2249,7 +1999,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>45</v>
       </c>
@@ -2260,7 +2010,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>45</v>
       </c>
@@ -2271,7 +2021,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>45</v>
       </c>
@@ -2282,7 +2032,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>45</v>
       </c>
@@ -2293,7 +2043,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>45</v>
       </c>
@@ -2313,9 +2063,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E9ECB9-9509-4435-9143-07DA83ABD06A}">
   <dimension ref="B2:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -2326,7 +2076,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>59</v>
       </c>
@@ -2337,7 +2087,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>59</v>
       </c>
@@ -2348,7 +2098,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>59</v>
       </c>
@@ -2359,7 +2109,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>59</v>
       </c>
@@ -2370,7 +2120,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>59</v>
       </c>
@@ -2381,7 +2131,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>59</v>
       </c>
@@ -2392,7 +2142,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>59</v>
       </c>
@@ -2403,7 +2153,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>59</v>
       </c>
@@ -2414,7 +2164,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>59</v>
       </c>
@@ -2425,7 +2175,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B12" s="5" t="s">
         <v>59</v>
       </c>
@@ -2436,7 +2186,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>59</v>
       </c>
@@ -2447,7 +2197,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>59</v>
       </c>
@@ -2458,7 +2208,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>59</v>
       </c>
@@ -2469,7 +2219,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>59</v>
       </c>
@@ -2488,12 +2238,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9318431B-ADA9-43B9-8F56-BA9994346673}">
   <dimension ref="B1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="206.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="206.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B1" s="11" t="s">
         <v>46</v>
       </c>
@@ -2504,7 +2254,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="12" t="s">
         <v>59</v>
       </c>
@@ -2515,7 +2265,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="12" t="s">
         <v>59</v>
       </c>
@@ -2526,7 +2276,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="12" t="s">
         <v>59</v>
       </c>
@@ -2537,7 +2287,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="12" t="s">
         <v>59</v>
       </c>
@@ -2548,7 +2298,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
         <v>59</v>
       </c>
@@ -2559,7 +2309,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
         <v>59</v>
       </c>
@@ -2570,7 +2320,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="8" t="s">
         <v>45</v>
       </c>
@@ -2581,7 +2331,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
         <v>59</v>
       </c>
@@ -2592,7 +2342,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
         <v>59</v>
       </c>
@@ -2603,7 +2353,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B11" s="8" t="s">
         <v>45</v>
       </c>
@@ -2614,7 +2364,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B12" s="8" t="s">
         <v>45</v>
       </c>
@@ -2625,7 +2375,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="8" t="s">
         <v>45</v>
       </c>
@@ -2636,7 +2386,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="12" t="s">
         <v>59</v>
       </c>
@@ -2647,7 +2397,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="8" t="s">
         <v>45</v>
       </c>
@@ -2658,7 +2408,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B16" s="8" t="s">
         <v>45</v>
       </c>
@@ -2669,7 +2419,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B17" s="8" t="s">
         <v>45</v>
       </c>
@@ -2680,7 +2430,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
         <v>59</v>
       </c>
@@ -2691,7 +2441,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
         <v>59</v>
       </c>
@@ -2702,7 +2452,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B20" s="12" t="s">
         <v>59</v>
       </c>
@@ -2713,7 +2463,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B21" s="12" t="s">
         <v>59</v>
       </c>
@@ -2724,7 +2474,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B22" s="12" t="s">
         <v>59</v>
       </c>
@@ -2748,18 +2498,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A2924F0-1E35-4E1D-BB63-0CAF182B060F}">
   <dimension ref="A1:M48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="87.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="87.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>176</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>44</v>
@@ -2770,603 +2521,726 @@
       <c r="D1" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E1" s="20" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E2" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="E3" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="E5" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="C6" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="E6" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="C7" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="D8" s="21" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="E8" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B9" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="C9" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="43.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="E15" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="C16" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="E16" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="C17" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B10" s="2" t="s">
+      <c r="E17" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="41.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="C18" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="E18" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>135</v>
+      <c r="E19" s="1" t="s">
+        <v>175</v>
       </c>
       <c r="J19" s="1"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="B20" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>135</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>175</v>
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="1" t="s">
         <v>135</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>175</v>
       </c>
       <c r="J21" s="1"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="B22" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>135</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>175</v>
       </c>
       <c r="J22" s="1"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="B23" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D24" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="E24" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D25" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C25" s="2" t="s">
+      <c r="E25" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D26" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="E26" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D27" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C27" s="2" t="s">
+      <c r="E27" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D29" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="E29" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="D29" s="2" t="s">
+      <c r="E30" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D30" s="2" t="s">
+      <c r="E31" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="E32" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="C33" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="D32" s="2" t="s">
+      <c r="E33" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E34" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D35" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E35" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B36" s="21" t="s">
-        <v>171</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="B36" s="22" t="s">
         <v>170</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="C36" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E36" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D37" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E37" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D38" s="2" t="s">
+      <c r="D38" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E38" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C39" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="D39" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E39" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="D40" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E40" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B41" s="20" t="s">
-        <v>166</v>
-      </c>
-      <c r="C41" s="2" t="s">
+      <c r="B41" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="C41" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="45" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E41" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="45" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1"/>
       <c r="B48" s="2"/>
       <c r="C48" s="1"/>
@@ -3378,158 +3252,13 @@
       <sortCondition ref="B1:B48"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="J19:M22 A29:A35 A45:D48 A36:B41 D29:D41 C26:C27 C30:C31 C34:C35 C38:C39 A2:D3 C18:C19 C6:C7 C22:C23 C10:C11 C14:C15">
-    <cfRule type="cellIs" dxfId="30" priority="36" operator="equal">
+  <conditionalFormatting sqref="A2:E41">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:B4 D4">
-    <cfRule type="cellIs" dxfId="29" priority="34" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:B5 D5">
-    <cfRule type="cellIs" dxfId="28" priority="33" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6:B6 D6">
-    <cfRule type="cellIs" dxfId="27" priority="32" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A7:B7 D7">
-    <cfRule type="cellIs" dxfId="26" priority="31" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A8:B8 D8">
-    <cfRule type="cellIs" dxfId="25" priority="30" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A9:B9 D9">
-    <cfRule type="cellIs" dxfId="24" priority="29" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A10:B10 D10">
-    <cfRule type="cellIs" dxfId="23" priority="28" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A11:B11 D11">
-    <cfRule type="cellIs" dxfId="22" priority="27" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A12:B12 D12">
-    <cfRule type="cellIs" dxfId="21" priority="26" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A13:B13 D13">
-    <cfRule type="cellIs" dxfId="20" priority="25" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A14:B14 D14">
-    <cfRule type="cellIs" dxfId="19" priority="24" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A15:B15 D15">
-    <cfRule type="cellIs" dxfId="18" priority="23" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A16:B16 D16">
-    <cfRule type="cellIs" dxfId="17" priority="22" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A17:B17 D17">
-    <cfRule type="cellIs" dxfId="16" priority="21" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A18:B18 D18">
-    <cfRule type="cellIs" dxfId="15" priority="20" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A19:B19 D19">
-    <cfRule type="cellIs" dxfId="14" priority="19" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A20:B20 D20">
-    <cfRule type="cellIs" dxfId="13" priority="18" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A21:B21 D21">
-    <cfRule type="cellIs" dxfId="12" priority="17" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A22:B22 D22">
-    <cfRule type="cellIs" dxfId="11" priority="16" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A23:B23 D23">
-    <cfRule type="cellIs" dxfId="10" priority="15" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A24:B24 D24">
-    <cfRule type="cellIs" dxfId="9" priority="14" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A25:B25 D25">
-    <cfRule type="cellIs" dxfId="8" priority="13" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A26:B26 D26">
-    <cfRule type="cellIs" dxfId="7" priority="12" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A27:B27 D27">
-    <cfRule type="cellIs" dxfId="6" priority="11" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A28:B28 D28">
-    <cfRule type="cellIs" dxfId="5" priority="10" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B29:B35">
-    <cfRule type="cellIs" dxfId="4" priority="7" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C28 C32 C36 C40">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C29 C33 C37 C41">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C4 C20 C8 C24 C12 C16">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C5 C21 C9 C25 C13 C17">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+  <conditionalFormatting sqref="J19:M22 A45:D48">
+    <cfRule type="cellIs" dxfId="0" priority="37" operator="equal">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3540,12 +3269,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BE193EC-6A88-4F24-8FA9-C3B527D61F00}">
   <dimension ref="B2:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="41.42578125" customWidth="1"/>
+    <col min="2" max="2" width="41.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:3" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B2" s="19" t="s">
         <v>123</v>
       </c>
@@ -3553,7 +3282,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="173.25" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B3" s="19" t="s">
         <v>124</v>
       </c>
@@ -3561,27 +3290,27 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="63" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="19" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="299.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" ht="62.4" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" ht="93.6" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="204.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:3" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:3" ht="109.2" x14ac:dyDescent="0.3">
       <c r="B8" s="19" t="s">
         <v>129</v>
       </c>

</xml_diff>

<commit_message>
preliminares del 17 de octubre
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES 2.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF6F658-FC35-45DA-A962-0D847F5E8D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838BBE56-4B24-43BD-A594-1571E9F0A18B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="86220" yWindow="-150" windowWidth="19635" windowHeight="21285" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1284,15 +1284,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1306,7 +1306,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1320,7 +1320,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1334,7 +1334,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" ht="43" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1376,7 +1376,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -1404,7 +1404,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -1432,7 +1432,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>1</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1502,7 +1502,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -1516,7 +1516,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" ht="43" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>20</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>22</v>
       </c>
@@ -1544,7 +1544,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
         <v>1</v>
       </c>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>33</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>4</v>
       </c>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
@@ -1641,12 +1641,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8E058B-C30B-45F0-BBCF-B7D4D02421F4}">
   <dimension ref="B2:L12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="8" max="8" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>83</v>
       </c>
@@ -1678,7 +1678,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>88</v>
       </c>
@@ -1710,7 +1710,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="18" t="s">
         <v>90</v>
       </c>
@@ -1742,7 +1742,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>92</v>
       </c>
@@ -1774,7 +1774,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>101</v>
       </c>
@@ -1806,7 +1806,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>95</v>
       </c>
@@ -1838,7 +1838,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="17" t="s">
         <v>97</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>99</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="H10" s="18" t="s">
         <v>117</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="H11" t="s">
         <v>119</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="H12" t="s">
         <v>119</v>
       </c>
@@ -1961,12 +1961,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CD9C86-BB81-45D2-B52F-9BBB3BE4D29C}">
   <dimension ref="B2:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="46.5546875" customWidth="1"/>
+    <col min="4" max="4" width="46.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -1977,7 +1977,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="5" t="s">
         <v>45</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>45</v>
       </c>
@@ -1999,7 +1999,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B5" s="5" t="s">
         <v>45</v>
       </c>
@@ -2010,7 +2010,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B6" s="5" t="s">
         <v>45</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B7" s="5" t="s">
         <v>45</v>
       </c>
@@ -2032,7 +2032,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B8" s="5" t="s">
         <v>45</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B9" s="5" t="s">
         <v>45</v>
       </c>
@@ -2063,9 +2063,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E9ECB9-9509-4435-9143-07DA83ABD06A}">
   <dimension ref="B2:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B3" s="5" t="s">
         <v>59</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B4" s="5" t="s">
         <v>59</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B5" s="5" t="s">
         <v>59</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B6" s="5" t="s">
         <v>59</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B7" s="5" t="s">
         <v>59</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B8" s="5" t="s">
         <v>59</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B9" s="5" t="s">
         <v>59</v>
       </c>
@@ -2153,7 +2153,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B10" s="5" t="s">
         <v>59</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B11" s="5" t="s">
         <v>59</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B12" s="5" t="s">
         <v>59</v>
       </c>
@@ -2186,7 +2186,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B13" s="5" t="s">
         <v>59</v>
       </c>
@@ -2197,7 +2197,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B14" s="5" t="s">
         <v>59</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B15" s="5" t="s">
         <v>59</v>
       </c>
@@ -2219,7 +2219,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B16" s="5" t="s">
         <v>59</v>
       </c>
@@ -2238,12 +2238,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9318431B-ADA9-43B9-8F56-BA9994346673}">
   <dimension ref="B1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="206.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="206.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B1" s="11" t="s">
         <v>46</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B2" s="12" t="s">
         <v>59</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B3" s="12" t="s">
         <v>59</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B4" s="12" t="s">
         <v>59</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B5" s="12" t="s">
         <v>59</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B6" s="12" t="s">
         <v>59</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B7" s="12" t="s">
         <v>59</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B8" s="8" t="s">
         <v>45</v>
       </c>
@@ -2331,7 +2331,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B9" s="12" t="s">
         <v>59</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B10" s="12" t="s">
         <v>59</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B11" s="8" t="s">
         <v>45</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B12" s="8" t="s">
         <v>45</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B13" s="8" t="s">
         <v>45</v>
       </c>
@@ -2386,7 +2386,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" ht="16" x14ac:dyDescent="0.4">
       <c r="B14" s="12" t="s">
         <v>59</v>
       </c>
@@ -2397,7 +2397,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B15" s="8" t="s">
         <v>45</v>
       </c>
@@ -2408,7 +2408,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B16" s="8" t="s">
         <v>45</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B17" s="8" t="s">
         <v>45</v>
       </c>
@@ -2430,7 +2430,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B18" s="12" t="s">
         <v>59</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B19" s="12" t="s">
         <v>59</v>
       </c>
@@ -2452,7 +2452,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B20" s="12" t="s">
         <v>59</v>
       </c>
@@ -2463,7 +2463,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B21" s="12" t="s">
         <v>59</v>
       </c>
@@ -2474,7 +2474,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:4" ht="16" x14ac:dyDescent="0.35">
       <c r="B22" s="12" t="s">
         <v>59</v>
       </c>
@@ -2498,17 +2498,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A2924F0-1E35-4E1D-BB63-0CAF182B060F}">
   <dimension ref="A1:M48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="87.6640625" customWidth="1"/>
+    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7265625" customWidth="1"/>
+    <col min="12" max="12" width="87.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>176</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>133</v>
       </c>
@@ -2542,7 +2542,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>133</v>
       </c>
@@ -2559,7 +2559,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="21" t="s">
         <v>133</v>
       </c>
@@ -2576,41 +2576,41 @@
         <v>175</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B5" s="1" t="s">
+    <row r="5" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c r="D5" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D6" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="21" t="s">
         <v>133</v>
       </c>
@@ -2627,7 +2627,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="21" t="s">
         <v>133</v>
       </c>
@@ -2638,13 +2638,13 @@
         <v>140</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="E8" s="21" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="21" t="s">
         <v>133</v>
       </c>
@@ -2661,7 +2661,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="21" t="s">
         <v>133</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="27.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="21" t="s">
         <v>133</v>
       </c>
@@ -2695,7 +2695,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="21" t="s">
         <v>133</v>
       </c>
@@ -2712,7 +2712,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="21" t="s">
         <v>133</v>
       </c>
@@ -2729,7 +2729,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="43.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="21" t="s">
         <v>133</v>
       </c>
@@ -2746,58 +2746,58 @@
         <v>175</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B15" s="1" t="s">
+    <row r="15" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B15" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B16" s="1" t="s">
+      <c r="D15" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B17" s="1" t="s">
+      <c r="D16" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B17" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="41.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D17" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="41.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>133</v>
       </c>
@@ -2814,20 +2814,20 @@
         <v>175</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B19" s="1" t="s">
+    <row r="19" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="D19" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E19" s="21" t="s">
         <v>175</v>
       </c>
       <c r="J19" s="1"/>
@@ -2835,20 +2835,20 @@
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B20" s="1" t="s">
+    <row r="20" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E20" s="1" t="s">
+      <c r="D20" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E20" s="21" t="s">
         <v>175</v>
       </c>
       <c r="J20" s="1"/>
@@ -2856,7 +2856,7 @@
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>133</v>
       </c>
@@ -2877,7 +2877,7 @@
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>133</v>
       </c>
@@ -2898,7 +2898,7 @@
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>133</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>133</v>
       </c>
@@ -2932,7 +2932,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>133</v>
       </c>
@@ -2949,7 +2949,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
         <v>133</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>133</v>
       </c>
@@ -2983,7 +2983,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
         <v>133</v>
       </c>
@@ -3000,7 +3000,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>133</v>
       </c>
@@ -3017,7 +3017,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>133</v>
       </c>
@@ -3034,7 +3034,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>133</v>
       </c>
@@ -3051,7 +3051,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>133</v>
       </c>
@@ -3068,7 +3068,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
         <v>133</v>
       </c>
@@ -3085,7 +3085,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>133</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>4</v>
       </c>
@@ -3119,7 +3119,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
         <v>133</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
         <v>38</v>
       </c>
@@ -3153,7 +3153,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="1" t="s">
         <v>133</v>
       </c>
@@ -3170,7 +3170,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="1" t="s">
         <v>9</v>
       </c>
@@ -3187,7 +3187,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
         <v>4</v>
       </c>
@@ -3204,7 +3204,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
         <v>133</v>
       </c>
@@ -3221,26 +3221,26 @@
         <v>175</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="45" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="45" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="1"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="1"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="1"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="1"/>
       <c r="B48" s="2"/>
       <c r="C48" s="1"/>
@@ -3269,12 +3269,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BE193EC-6A88-4F24-8FA9-C3B527D61F00}">
   <dimension ref="B2:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="41.44140625" customWidth="1"/>
+    <col min="2" max="2" width="41.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" ht="32" x14ac:dyDescent="0.35">
       <c r="B2" s="19" t="s">
         <v>123</v>
       </c>
@@ -3282,7 +3282,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" ht="48" x14ac:dyDescent="0.35">
       <c r="B3" s="19" t="s">
         <v>124</v>
       </c>
@@ -3290,27 +3290,27 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" ht="16" x14ac:dyDescent="0.35">
       <c r="B4" s="19" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" ht="64" x14ac:dyDescent="0.35">
       <c r="B5" s="19" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" ht="96" x14ac:dyDescent="0.35">
       <c r="B6" s="19" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" ht="48" x14ac:dyDescent="0.35">
       <c r="B7" s="19" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" ht="112" x14ac:dyDescent="0.35">
       <c r="B8" s="19" t="s">
         <v>129</v>
       </c>

</xml_diff>

<commit_message>
Correcciones para las referencias
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES 2.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES 2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838BBE56-4B24-43BD-A594-1571E9F0A18B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA70B49-B10F-4E0F-B3B2-EDCE38094A57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="86220" yWindow="-150" windowWidth="19635" windowHeight="21285" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Hoja4!$B$1:$D$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Hoja6!$A$1:$D$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Hoja6!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="179">
   <si>
     <t>Director(es) que lo solicita</t>
   </si>
@@ -574,9 +574,6 @@
     <t>Dra. Adri</t>
   </si>
   <si>
-    <t>Seccipon 1.1. Cambiar el ejemplo de la genomica por ser muy especifico</t>
-  </si>
-  <si>
     <t>Pendiente</t>
   </si>
   <si>
@@ -707,6 +704,9 @@
   </si>
   <si>
     <t>LISTO</t>
+  </si>
+  <si>
+    <t>Seccion 1.1. Cambiar el ejemplo de la genomica por ser muy especifico</t>
   </si>
 </sst>
 </file>
@@ -941,11 +941,11 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2510,7 +2510,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>44</v>
@@ -2522,40 +2522,40 @@
         <v>76</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="A2" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B2" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="C2" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D2" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="E2" s="21" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="A3" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="E3" s="21" t="s">
         <v>174</v>
       </c>
     </row>
@@ -2564,19 +2564,19 @@
         <v>133</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="21" t="s">
         <v>133</v>
       </c>
@@ -2584,16 +2584,16 @@
         <v>19</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="21" t="s">
         <v>133</v>
       </c>
@@ -2601,13 +2601,13 @@
         <v>19</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2618,13 +2618,13 @@
         <v>19</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -2635,13 +2635,13 @@
         <v>19</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>140</v>
+        <v>176</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2655,13 +2655,13 @@
         <v>141</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="21" t="s">
         <v>133</v>
       </c>
@@ -2669,13 +2669,13 @@
         <v>19</v>
       </c>
       <c r="C10" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="D10" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="D10" s="21" t="s">
-        <v>178</v>
-      </c>
       <c r="E10" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="27.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -2686,13 +2686,13 @@
         <v>19</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2703,16 +2703,16 @@
         <v>19</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="21" t="s">
         <v>133</v>
       </c>
@@ -2720,13 +2720,13 @@
         <v>19</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -2737,16 +2737,16 @@
         <v>19</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="21" t="s">
         <v>133</v>
       </c>
@@ -2754,13 +2754,13 @@
         <v>19</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2768,16 +2768,16 @@
         <v>133</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>19</v>
+        <v>148</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2785,33 +2785,33 @@
         <v>133</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>19</v>
+        <v>148</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="41.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>175</v>
+      <c r="A18" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2819,16 +2819,16 @@
         <v>133</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J19" s="1"/>
       <c r="K19" s="2"/>
@@ -2840,16 +2840,16 @@
         <v>133</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E20" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="2"/>
@@ -2857,20 +2857,20 @@
       <c r="M20" s="2"/>
     </row>
     <row r="21" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>175</v>
+      <c r="A21" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>174</v>
       </c>
       <c r="J21" s="1"/>
       <c r="K21" s="2"/>
@@ -2878,20 +2878,20 @@
       <c r="M21" s="2"/>
     </row>
     <row r="22" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>175</v>
+      <c r="A22" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>174</v>
       </c>
       <c r="J22" s="1"/>
       <c r="K22" s="2"/>
@@ -2899,71 +2899,71 @@
       <c r="M22" s="2"/>
     </row>
     <row r="23" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="A23" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="E23" s="21" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="C24" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>175</v>
+      <c r="D24" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="E24" s="21" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>175</v>
+      <c r="A25" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>159</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="E25" s="21" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="E26" s="21" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2971,67 +2971,67 @@
         <v>133</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>152</v>
+        <v>8</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>152</v>
+        <v>8</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>152</v>
+        <v>19</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>160</v>
+        <v>132</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>161</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -3039,16 +3039,16 @@
         <v>133</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -3056,16 +3056,16 @@
         <v>133</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>166</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -3073,152 +3073,135 @@
         <v>133</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>167</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
-        <v>133</v>
+        <v>4</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>163</v>
+        <v>32</v>
       </c>
       <c r="C34" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B35" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="D34" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="1" t="s">
+      <c r="D35" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B36" s="22" t="s">
-        <v>170</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="B39" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>37</v>
+        <v>133</v>
+      </c>
+      <c r="B40" s="22" t="s">
+        <v>164</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>36</v>
+        <v>163</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B41" s="23" t="s">
-        <v>165</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -3247,12 +3230,12 @@
       <c r="D48" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D48" xr:uid="{2A2924F0-1E35-4E1D-BB63-0CAF182B060F}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D48">
-      <sortCondition ref="B1:B48"/>
+  <autoFilter ref="A1:E1" xr:uid="{2A2924F0-1E35-4E1D-BB63-0CAF182B060F}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E40">
+      <sortCondition ref="D1"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="A2:E41">
+  <conditionalFormatting sqref="A2:E40">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>#REF!</formula>
     </cfRule>

</xml_diff>

<commit_message>
Correcciones de citas y caracterización de casos
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES 2.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES 2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA70B49-B10F-4E0F-B3B2-EDCE38094A57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D959C7-8AF5-410C-9264-94D4806D3B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -888,7 +888,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -941,7 +941,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1284,15 +1287,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.453125" customWidth="1"/>
+    <col min="3" max="3" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1306,7 +1309,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1320,7 +1323,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1334,7 +1337,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1348,7 +1351,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1362,7 +1365,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="43" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1376,7 +1379,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -1390,7 +1393,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -1404,7 +1407,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -1418,7 +1421,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -1432,7 +1435,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1446,7 +1449,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -1460,7 +1463,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>1</v>
       </c>
@@ -1474,7 +1477,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -1488,7 +1491,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1502,7 +1505,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -1516,7 +1519,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="43" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>20</v>
       </c>
@@ -1530,7 +1533,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>22</v>
       </c>
@@ -1544,7 +1547,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>1</v>
       </c>
@@ -1556,7 +1559,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>33</v>
       </c>
@@ -1570,7 +1573,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1582,7 +1585,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>4</v>
       </c>
@@ -1594,7 +1597,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -1606,7 +1609,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:4" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
@@ -1641,12 +1644,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8E058B-C30B-45F0-BBCF-B7D4D02421F4}">
   <dimension ref="B2:L12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="8" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>83</v>
       </c>
@@ -1678,7 +1681,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>88</v>
       </c>
@@ -1710,7 +1713,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="18" t="s">
         <v>90</v>
       </c>
@@ -1742,7 +1745,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" ht="30" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>92</v>
       </c>
@@ -1774,7 +1777,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>101</v>
       </c>
@@ -1806,7 +1809,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>95</v>
       </c>
@@ -1838,7 +1841,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="17" t="s">
         <v>97</v>
       </c>
@@ -1870,7 +1873,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>99</v>
       </c>
@@ -1902,7 +1905,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H10" s="18" t="s">
         <v>117</v>
       </c>
@@ -1919,7 +1922,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H11" t="s">
         <v>119</v>
       </c>
@@ -1936,7 +1939,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H12" t="s">
         <v>119</v>
       </c>
@@ -1961,12 +1964,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CD9C86-BB81-45D2-B52F-9BBB3BE4D29C}">
   <dimension ref="B2:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="46.54296875" customWidth="1"/>
+    <col min="4" max="4" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -1977,7 +1980,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>45</v>
       </c>
@@ -1988,7 +1991,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>45</v>
       </c>
@@ -1999,7 +2002,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>45</v>
       </c>
@@ -2010,7 +2013,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>45</v>
       </c>
@@ -2021,7 +2024,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
         <v>45</v>
       </c>
@@ -2032,7 +2035,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>45</v>
       </c>
@@ -2043,7 +2046,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>45</v>
       </c>
@@ -2063,9 +2066,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E9ECB9-9509-4435-9143-07DA83ABD06A}">
   <dimension ref="B2:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -2076,7 +2079,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>59</v>
       </c>
@@ -2087,7 +2090,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>59</v>
       </c>
@@ -2098,7 +2101,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>59</v>
       </c>
@@ -2109,7 +2112,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>59</v>
       </c>
@@ -2120,7 +2123,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
         <v>59</v>
       </c>
@@ -2131,7 +2134,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>59</v>
       </c>
@@ -2142,7 +2145,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>59</v>
       </c>
@@ -2153,7 +2156,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="5" t="s">
         <v>59</v>
       </c>
@@ -2164,7 +2167,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="5" t="s">
         <v>59</v>
       </c>
@@ -2175,7 +2178,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="5" t="s">
         <v>59</v>
       </c>
@@ -2186,7 +2189,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="5" t="s">
         <v>59</v>
       </c>
@@ -2197,7 +2200,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
         <v>59</v>
       </c>
@@ -2208,7 +2211,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>59</v>
       </c>
@@ -2219,7 +2222,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>59</v>
       </c>
@@ -2238,12 +2241,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9318431B-ADA9-43B9-8F56-BA9994346673}">
   <dimension ref="B1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="206.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="206.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" s="11" t="s">
         <v>46</v>
       </c>
@@ -2254,7 +2257,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
         <v>59</v>
       </c>
@@ -2265,7 +2268,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="12" t="s">
         <v>59</v>
       </c>
@@ -2276,7 +2279,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="12" t="s">
         <v>59</v>
       </c>
@@ -2287,7 +2290,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
         <v>59</v>
       </c>
@@ -2298,7 +2301,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
         <v>59</v>
       </c>
@@ -2309,7 +2312,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
         <v>59</v>
       </c>
@@ -2320,7 +2323,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
         <v>45</v>
       </c>
@@ -2331,7 +2334,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>59</v>
       </c>
@@ -2342,7 +2345,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
         <v>59</v>
       </c>
@@ -2353,7 +2356,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
         <v>45</v>
       </c>
@@ -2364,7 +2367,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>45</v>
       </c>
@@ -2375,7 +2378,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>45</v>
       </c>
@@ -2386,7 +2389,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="16" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
         <v>59</v>
       </c>
@@ -2397,7 +2400,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
         <v>45</v>
       </c>
@@ -2408,7 +2411,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
         <v>45</v>
       </c>
@@ -2419,7 +2422,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
         <v>45</v>
       </c>
@@ -2430,7 +2433,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
         <v>59</v>
       </c>
@@ -2441,7 +2444,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
         <v>59</v>
       </c>
@@ -2452,7 +2455,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
         <v>59</v>
       </c>
@@ -2463,7 +2466,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
         <v>59</v>
       </c>
@@ -2474,7 +2477,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
         <v>59</v>
       </c>
@@ -2498,17 +2501,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A2924F0-1E35-4E1D-BB63-0CAF182B060F}">
   <dimension ref="A1:M48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.7265625" customWidth="1"/>
-    <col min="12" max="12" width="87.7265625" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="12" max="12" width="87.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>175</v>
       </c>
@@ -2525,7 +2528,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
         <v>133</v>
       </c>
@@ -2542,7 +2545,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
         <v>133</v>
       </c>
@@ -2559,7 +2562,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>133</v>
       </c>
@@ -2576,7 +2579,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
         <v>133</v>
       </c>
@@ -2593,7 +2596,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
         <v>133</v>
       </c>
@@ -2610,7 +2613,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
         <v>133</v>
       </c>
@@ -2627,7 +2630,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="21" t="s">
         <v>133</v>
       </c>
@@ -2644,7 +2647,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
         <v>133</v>
       </c>
@@ -2661,7 +2664,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
         <v>133</v>
       </c>
@@ -2678,7 +2681,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="27.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
         <v>133</v>
       </c>
@@ -2695,7 +2698,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
         <v>133</v>
       </c>
@@ -2712,7 +2715,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
         <v>133</v>
       </c>
@@ -2729,7 +2732,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="21" t="s">
         <v>133</v>
       </c>
@@ -2746,7 +2749,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
         <v>133</v>
       </c>
@@ -2763,7 +2766,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>133</v>
       </c>
@@ -2780,7 +2783,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:13" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
         <v>133</v>
       </c>
@@ -2797,7 +2800,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="41.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:13" ht="41.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="21" t="s">
         <v>133</v>
       </c>
@@ -2814,7 +2817,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="21" t="s">
         <v>133</v>
       </c>
@@ -2835,7 +2838,7 @@
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="21" t="s">
         <v>133</v>
       </c>
@@ -2856,7 +2859,7 @@
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="21" t="s">
         <v>133</v>
       </c>
@@ -2877,7 +2880,7 @@
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="21" t="s">
         <v>133</v>
       </c>
@@ -2898,7 +2901,7 @@
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="21" t="s">
         <v>133</v>
       </c>
@@ -2915,7 +2918,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="21" t="s">
         <v>133</v>
       </c>
@@ -2932,7 +2935,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="21" t="s">
         <v>133</v>
       </c>
@@ -2949,7 +2952,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:13" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
         <v>133</v>
       </c>
@@ -2966,83 +2969,83 @@
         <v>174</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B27" s="1" t="s">
+    <row r="27" spans="1:13" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="D27" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>161</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C29" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>134</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>162</v>
+        <v>8</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>134</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>162</v>
+        <v>19</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>165</v>
+        <v>132</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>134</v>
@@ -3051,7 +3054,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>133</v>
       </c>
@@ -3059,7 +3062,7 @@
         <v>162</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>134</v>
@@ -3068,7 +3071,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>133</v>
       </c>
@@ -3076,7 +3079,7 @@
         <v>162</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>134</v>
@@ -3085,15 +3088,15 @@
         <v>174</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>4</v>
+        <v>133</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>32</v>
+        <v>162</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>35</v>
+        <v>167</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>134</v>
@@ -3102,15 +3105,15 @@
         <v>174</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B35" s="23" t="s">
-        <v>169</v>
+        <v>4</v>
+      </c>
+      <c r="B35" s="24" t="s">
+        <v>32</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>168</v>
+        <v>35</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>134</v>
@@ -3119,15 +3122,15 @@
         <v>174</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>38</v>
+        <v>133</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>40</v>
+        <v>169</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>39</v>
+        <v>168</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>134</v>
@@ -3136,15 +3139,15 @@
         <v>174</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>133</v>
+        <v>38</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>170</v>
+        <v>40</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>171</v>
+        <v>39</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>134</v>
@@ -3153,15 +3156,15 @@
         <v>174</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>9</v>
+        <v>133</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>42</v>
+        <v>170</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>41</v>
+        <v>171</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>134</v>
@@ -3170,15 +3173,15 @@
         <v>174</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>134</v>
@@ -3187,15 +3190,15 @@
         <v>174</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B40" s="22" t="s">
-        <v>164</v>
+        <v>4</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>163</v>
+        <v>36</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>134</v>
@@ -3204,26 +3207,26 @@
         <v>174</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="45" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="2"/>
       <c r="C48" s="1"/>
@@ -3252,12 +3255,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BE193EC-6A88-4F24-8FA9-C3B527D61F00}">
   <dimension ref="B2:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="41.453125" customWidth="1"/>
+    <col min="2" max="2" width="41.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="32" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:3" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B2" s="19" t="s">
         <v>123</v>
       </c>
@@ -3265,7 +3268,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="48" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:3" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B3" s="19" t="s">
         <v>124</v>
       </c>
@@ -3273,27 +3276,27 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="16" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="19" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="64" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" ht="63" x14ac:dyDescent="0.25">
       <c r="B5" s="19" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="96" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" ht="94.5" x14ac:dyDescent="0.25">
       <c r="B6" s="19" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="48" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B7" s="19" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="112" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:3" ht="110.25" x14ac:dyDescent="0.25">
       <c r="B8" s="19" t="s">
         <v>129</v>
       </c>

</xml_diff>